<commit_message>
fixed tests for 2026 categories
</commit_message>
<xml_diff>
--- a/owlcms/src/test/resources/testData/missingCellsRegistration.xlsx
+++ b/owlcms/src/test/resources/testData/missingCellsRegistration.xlsx
@@ -539,7 +539,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>U13 M 42</t>
+          <t>U13 M 45</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>M45 94</t>
+          <t>M45 95</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">

</xml_diff>